<commit_message>
Update 001 - 092625 - Deges Master Ability Cross Reference Matrix.xlsx
Updated Ability x ref
</commit_message>
<xml_diff>
--- a/001 - 092625 - Deges Master Ability Cross Reference Matrix.xlsx
+++ b/001 - 092625 - Deges Master Ability Cross Reference Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JayAppell\Documents\GitHub\HouseRulesGuide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E6C51C-F3F3-4534-BD90-4A5693C885F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8574C73E-5D6A-43C2-8D38-58F22FF2AFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60705" yWindow="1365" windowWidth="28800" windowHeight="15375" xr2:uid="{2732B8C7-4FC7-48F8-9848-8F5EC97AA8E5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{2732B8C7-4FC7-48F8-9848-8F5EC97AA8E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="712">
   <si>
     <t>Ability Name</t>
   </si>
@@ -2185,14 +2185,20 @@
     <t>Use Arrow</t>
   </si>
   <si>
-    <t>092025 - 2225</t>
+    <t>9/27 Use on Reign of Madness Boss Map – Puts down 3 walls </t>
+  </si>
+  <si>
+    <t>092725 - 2308</t>
+  </si>
+  <si>
+    <t>&lt;-----------------------------------</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2286,8 +2292,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F2328"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2300,8 +2320,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -2348,12 +2373,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2425,8 +2475,18 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -2760,12 +2820,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76B6FCBB-BF08-4DE4-A8BC-31BC55890723}">
-  <dimension ref="A1:E310"/>
+  <dimension ref="A1:J310"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.08984375" style="2" customWidth="1"/>
     <col min="2" max="3" width="30" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.08984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.54296875" style="4" customWidth="1"/>
     <col min="5" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
@@ -2776,7 +2836,7 @@
     </row>
     <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -4277,7 +4337,7 @@
       </c>
       <c r="D143" s="10"/>
     </row>
-    <row r="144" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="144" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B144" s="9" t="s">
         <v>126</v>
       </c>
@@ -4332,7 +4392,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="149" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="149" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B149" s="9" t="s">
         <v>129</v>
       </c>
@@ -5658,7 +5718,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="273" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="273" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B273" s="16" t="s">
         <v>225</v>
       </c>
@@ -5669,7 +5729,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="274" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="274" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B274" s="9" t="s">
         <v>357</v>
       </c>
@@ -5680,7 +5740,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="275" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="275" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B275" s="9" t="s">
         <v>288</v>
       </c>
@@ -5691,7 +5751,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="276" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="276" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B276" s="10" t="s">
         <v>226</v>
       </c>
@@ -5702,16 +5762,26 @@
         <v>703</v>
       </c>
     </row>
-    <row r="277" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="277" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B277" s="16" t="s">
         <v>227</v>
       </c>
       <c r="C277" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="D277" s="19"/>
-    </row>
-    <row r="278" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="D277" s="25" t="s">
+        <v>709</v>
+      </c>
+      <c r="E277" s="26" t="s">
+        <v>711</v>
+      </c>
+      <c r="F277" s="27"/>
+      <c r="G277" s="27"/>
+      <c r="H277" s="27"/>
+      <c r="I277" s="27"/>
+      <c r="J277" s="27"/>
+    </row>
+    <row r="278" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B278" s="16" t="s">
         <v>228</v>
       </c>
@@ -5720,7 +5790,7 @@
       </c>
       <c r="D278" s="19"/>
     </row>
-    <row r="279" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="279" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B279" s="9" t="s">
         <v>229</v>
       </c>
@@ -5731,7 +5801,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="280" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="280" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B280" s="9" t="s">
         <v>230</v>
       </c>
@@ -5742,7 +5812,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="281" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="281" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B281" s="9" t="s">
         <v>231</v>
       </c>
@@ -5753,7 +5823,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="282" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="282" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B282" s="12" t="s">
         <v>232</v>
       </c>
@@ -5764,7 +5834,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="283" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="283" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B283" s="12" t="s">
         <v>233</v>
       </c>
@@ -5773,7 +5843,7 @@
       </c>
       <c r="D283" s="19"/>
     </row>
-    <row r="284" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="284" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B284" s="9" t="s">
         <v>234</v>
       </c>
@@ -5784,7 +5854,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="285" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="285" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B285" s="9" t="s">
         <v>415</v>
       </c>
@@ -5795,7 +5865,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="286" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="286" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B286" s="9" t="s">
         <v>418</v>
       </c>
@@ -5806,7 +5876,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="287" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="287" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B287" s="9" t="s">
         <v>235</v>
       </c>
@@ -5817,7 +5887,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="288" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="288" spans="2:10" ht="29" x14ac:dyDescent="0.35">
       <c r="B288" s="9" t="s">
         <v>236</v>
       </c>
@@ -5934,7 +6004,7 @@
       </c>
       <c r="D298" s="10"/>
     </row>
-    <row r="299" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="299" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B299" s="9" t="s">
         <v>246</v>
       </c>
@@ -6032,7 +6102,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="308" spans="2:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="308" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B308" s="9" t="s">
         <v>254</v>
       </c>
@@ -6069,6 +6139,9 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D310">
     <sortCondition ref="B1:B310"/>
   </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="E277:J277"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="C133" r:id="rId1" display="https://demeo.fandom.com/wiki/Adamant_Potion" xr:uid="{E628E99E-77DC-4390-82D6-17D15C269584}"/>
   </hyperlinks>

</xml_diff>